<commit_message>
UpgradeBlock - GetStringWithUpgradeType 리팩터링
</commit_message>
<xml_diff>
--- a/Assets/Resources/DataBase/Upgrade Data/UpgradeDB.xlsx
+++ b/Assets/Resources/DataBase/Upgrade Data/UpgradeDB.xlsx
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>index</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -119,6 +119,14 @@
   </si>
   <si>
     <t>테스트 이름</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Add</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>안녕하세용</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -503,7 +511,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:V2"/>
+  <dimension ref="A1:V3"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="6.796875" customWidth="1"/>
@@ -647,6 +655,74 @@
         <v>15</v>
       </c>
     </row>
+    <row r="3" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3">
+        <v>9</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>2</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+      <c r="I3">
+        <v>3</v>
+      </c>
+      <c r="J3">
+        <v>3</v>
+      </c>
+      <c r="K3">
+        <v>4</v>
+      </c>
+      <c r="L3">
+        <v>4</v>
+      </c>
+      <c r="M3">
+        <v>5</v>
+      </c>
+      <c r="N3">
+        <v>5</v>
+      </c>
+      <c r="O3">
+        <v>6</v>
+      </c>
+      <c r="P3">
+        <v>6</v>
+      </c>
+      <c r="Q3">
+        <v>7</v>
+      </c>
+      <c r="R3">
+        <v>7</v>
+      </c>
+      <c r="S3">
+        <v>8</v>
+      </c>
+      <c r="T3">
+        <v>8</v>
+      </c>
+      <c r="U3">
+        <v>9</v>
+      </c>
+      <c r="V3">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>